<commit_message>
feat: fix status digitales matching, report exports, and docker deploy flow
</commit_message>
<xml_diff>
--- a/docs/excels/Data utilizada para importar tarjetas.xlsx
+++ b/docs/excels/Data utilizada para importar tarjetas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramse\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramse\Documents\Proyectos\celego\docs\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{1C5DB1DD-BFB3-45AA-B9D2-4E0FC227102E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{7FD18408-FC32-4DC9-AA45-D0D8FE51A0AD}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7FD18408-FC32-4DC9-AA45-D0D8FE51A0AD}"/>
   </bookViews>
   <sheets>
     <sheet name="IMPORTAR_DATA_DIARIA" sheetId="2" r:id="rId1"/>

</xml_diff>

<commit_message>
docs: guardar contexto operativo previo
</commit_message>
<xml_diff>
--- a/docs/excels/Data utilizada para importar tarjetas.xlsx
+++ b/docs/excels/Data utilizada para importar tarjetas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramse\Documents\Proyectos\celego\docs\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1C5DB1DD-BFB3-45AA-B9D2-4E0FC227102E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16A6215A-6FD4-4B38-A47B-F71501FEE81C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{7FD18408-FC32-4DC9-AA45-D0D8FE51A0AD}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="454">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1410" uniqueCount="455">
   <si>
     <t>EMISION</t>
   </si>
@@ -1402,6 +1402,9 @@
   <si>
     <t>j</t>
   </si>
+  <si>
+    <t>4921017885434644</t>
+  </si>
 </sst>
 </file>
 
@@ -2051,14 +2054,14 @@
       </c>
       <c r="B3" s="22">
         <f>COUNTIF(H:H,1)</f>
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
         <v>452</v>
       </c>
       <c r="F3">
         <f>B3</f>
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:36" x14ac:dyDescent="0.3">
@@ -6434,39 +6437,103 @@
       </c>
     </row>
     <row r="49" spans="1:33" x14ac:dyDescent="0.3">
-      <c r="A49" s="14"/>
-      <c r="B49" s="9"/>
+      <c r="A49" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B49" s="9">
+        <v>46135</v>
+      </c>
       <c r="C49" s="15"/>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-      <c r="F49" s="3"/>
-      <c r="G49" s="3"/>
-      <c r="H49" s="3"/>
-      <c r="I49" s="3"/>
-      <c r="J49" s="3"/>
-      <c r="K49" s="3"/>
-      <c r="L49" s="3"/>
-      <c r="M49" s="3"/>
-      <c r="N49" s="3"/>
-      <c r="O49" s="3"/>
-      <c r="P49" s="3"/>
-      <c r="Q49" s="3"/>
-      <c r="R49" s="3"/>
-      <c r="S49" s="3"/>
-      <c r="T49" s="3"/>
-      <c r="U49" s="3"/>
-      <c r="V49" s="3"/>
-      <c r="W49" s="3"/>
-      <c r="X49" s="3"/>
-      <c r="Y49" s="3"/>
-      <c r="Z49" s="3"/>
-      <c r="AA49" s="3"/>
-      <c r="AB49" s="3"/>
-      <c r="AC49" s="3"/>
-      <c r="AD49" s="3"/>
-      <c r="AE49" s="3"/>
-      <c r="AF49" s="3"/>
-      <c r="AG49" s="3"/>
+      <c r="D49" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="J49" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="K49" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="L49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="M49" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="N49" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="O49" s="3" t="s">
+        <v>410</v>
+      </c>
+      <c r="P49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="R49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="S49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="T49" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="U49" s="3" t="s">
+        <v>409</v>
+      </c>
+      <c r="V49" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="W49" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="X49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="Z49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AA49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AB49" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="AC49" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="AD49" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE49" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="AF49" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="AG49" s="3" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="50" spans="1:33" x14ac:dyDescent="0.3">
       <c r="A50" s="14"/>

</xml_diff>